<commit_message>
refactor(memo-45): update tracking table layout to single-line header and scale table to fit page
</commit_message>
<xml_diff>
--- a/frontend/static/docs/ขอส่งใบติดตามทวงถาม_45_วัน_Rebuild_Thai.xlsx
+++ b/frontend/static/docs/ขอส่งใบติดตามทวงถาม_45_วัน_Rebuild_Thai.xlsx
@@ -112,7 +112,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -891,7 +891,7 @@
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>ต.ค. ๕๗</t>
+          <t xml:space="preserve">          ต.ค. ๕๗</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -903,7 +903,7 @@
     <row r="20">
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>ต.ค. ๕๗</t>
+          <t xml:space="preserve">          ต.ค. ๕๗</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>มิ.ย. ๔๗</t>
+          <t xml:space="preserve">          มิ.ย. ๔๗</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -1100,7 +1100,7 @@
     <row r="17">
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>มิ.ย. ๔๗</t>
+          <t xml:space="preserve">          มิ.ย. ๔๗</t>
         </is>
       </c>
     </row>

</xml_diff>